<commit_message>
Refined cot and base prompting for category 2
</commit_message>
<xml_diff>
--- a/LLM_Extraction_and_CrossCritique/interactive-table/noteable_results/pipeline_comparison_p1_vs_p2.xlsx
+++ b/LLM_Extraction_and_CrossCritique/interactive-table/noteable_results/pipeline_comparison_p1_vs_p2.xlsx
@@ -834,10 +834,10 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J2">
-        <v>0.8888888888888888</v>
+        <v>0.7777777777777778</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -866,10 +866,10 @@
         <v>0</v>
       </c>
       <c r="I3">
+        <v>0.6</v>
+      </c>
+      <c r="J3">
         <v>0.6666666666666666</v>
-      </c>
-      <c r="J3">
-        <v>0.7407407407407408</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -898,10 +898,10 @@
         <v>0</v>
       </c>
       <c r="I4">
-        <v>1</v>
+        <v>0.7333333333333334</v>
       </c>
       <c r="J4">
-        <v>0.6666666666666666</v>
+        <v>0.8148148148148149</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -930,10 +930,10 @@
         <v>0</v>
       </c>
       <c r="I5">
-        <v>0.611111111111111</v>
+        <v>0.6</v>
       </c>
       <c r="J5">
-        <v>0.6296296296296297</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -956,10 +956,10 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I6">
         <v>0.5</v>
@@ -994,10 +994,10 @@
         <v>0</v>
       </c>
       <c r="I7">
-        <v>0.7777777777777778</v>
+        <v>0.6</v>
       </c>
       <c r="J7">
-        <v>0.7777777777777778</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1052,10 +1052,10 @@
         <v>0.8571428571428571</v>
       </c>
       <c r="G9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9">
         <v>0.6</v>
@@ -1090,7 +1090,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>0.7000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J10">
         <v>0.8571428571428571</v>
@@ -1116,16 +1116,16 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="G11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I11">
-        <v>0.2083333333333333</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="J11">
-        <v>0.2777777777777778</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1154,10 +1154,10 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>0.2666666666666667</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J12">
-        <v>0.3333333333333333</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1186,10 +1186,10 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>0.4333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="J13">
-        <v>0.5416666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1218,10 +1218,10 @@
         <v>0</v>
       </c>
       <c r="I14">
-        <v>0.4000000000000001</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J14">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1244,16 +1244,16 @@
         <v>0.75</v>
       </c>
       <c r="G15">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I15">
-        <v>0.4000000000000001</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="J15">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1308,16 +1308,16 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G17">
-        <v>0.1111111111111111</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>0.1111111111111111</v>
+        <v>0</v>
       </c>
       <c r="I17">
-        <v>0.5238095238095238</v>
+        <v>0.5</v>
       </c>
       <c r="J17">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1340,16 +1340,16 @@
         <v>0.875</v>
       </c>
       <c r="G18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I18">
-        <v>0.5416666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J18">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1372,10 +1372,10 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="G19">
-        <v>0.75</v>
+        <v>0.2</v>
       </c>
       <c r="H19">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="I19">
         <v>0.6</v>
@@ -1404,16 +1404,16 @@
         <v>0.625</v>
       </c>
       <c r="G20">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H20">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I20">
-        <v>0.6</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J20">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="21" spans="1:10">
@@ -1436,16 +1436,16 @@
         <v>0.625</v>
       </c>
       <c r="G21">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H21">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I21">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J21">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="22" spans="1:10">
@@ -1468,10 +1468,10 @@
         <v>0.625</v>
       </c>
       <c r="G22">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I22">
         <v>0.6</v>
@@ -1538,10 +1538,10 @@
         <v>0</v>
       </c>
       <c r="I24">
-        <v>0.5333333333333333</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J24">
-        <v>0.6666666666666666</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -1564,16 +1564,16 @@
         <v>0.75</v>
       </c>
       <c r="G25">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="H25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I25">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J25">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1596,10 +1596,10 @@
         <v>0.5</v>
       </c>
       <c r="G26">
-        <v>0.4444444444444444</v>
+        <v>0</v>
       </c>
       <c r="H26">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I26">
         <v>0.6</v>
@@ -1628,16 +1628,16 @@
         <v>0.625</v>
       </c>
       <c r="G27">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H27">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J27">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="28" spans="1:10">
@@ -1666,10 +1666,10 @@
         <v>0</v>
       </c>
       <c r="I28">
-        <v>0.4000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="J28">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -1692,16 +1692,16 @@
         <v>0.625</v>
       </c>
       <c r="G29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29">
-        <v>0.4000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="J29">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1724,10 +1724,10 @@
         <v>0.75</v>
       </c>
       <c r="G30">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I30">
         <v>0.5</v>
@@ -1756,16 +1756,16 @@
         <v>0.625</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I31">
-        <v>0.4000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="J31">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="32" spans="1:10">
@@ -1788,16 +1788,16 @@
         <v>0.75</v>
       </c>
       <c r="G32">
-        <v>0.8333333333333334</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I32">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J32">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1820,10 +1820,10 @@
         <v>0.75</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H33">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I33">
         <v>0.6</v>
@@ -1852,16 +1852,16 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="G34">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H34">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I34">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J34">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="35" spans="1:10">
@@ -1884,10 +1884,10 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="G35">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H35">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I35">
         <v>0.6</v>
@@ -1922,10 +1922,10 @@
         <v>0</v>
       </c>
       <c r="I36">
-        <v>0.5333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="J36">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -1954,10 +1954,10 @@
         <v>0</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J37">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="38" spans="1:10">
@@ -1986,10 +1986,10 @@
         <v>0</v>
       </c>
       <c r="I38">
-        <v>0.4333333333333333</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J38">
-        <v>0.5416666666666666</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="39" spans="1:10">
@@ -2012,13 +2012,13 @@
         <v>0.75</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I39">
-        <v>0.6666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J39">
         <v>0.75</v>
@@ -2044,16 +2044,16 @@
         <v>0.75</v>
       </c>
       <c r="G40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I40">
-        <v>0.5666666666666667</v>
+        <v>0.5</v>
       </c>
       <c r="J40">
-        <v>0.7083333333333334</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="41" spans="1:10">
@@ -2076,10 +2076,10 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41">
         <v>0.6</v>
@@ -2108,16 +2108,16 @@
         <v>0.75</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I42">
-        <v>0.5499999999999999</v>
+        <v>0.6</v>
       </c>
       <c r="J42">
-        <v>0.5833333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="43" spans="1:10">
@@ -2140,10 +2140,10 @@
         <v>0.75</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I43">
         <v>0.5</v>
@@ -2172,16 +2172,16 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="G44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I44">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="J44">
-        <v>0.75</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="45" spans="1:10">
@@ -2204,16 +2204,16 @@
         <v>0.5</v>
       </c>
       <c r="G45">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H45">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I45">
-        <v>0.5</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J45">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="46" spans="1:10">
@@ -2236,16 +2236,16 @@
         <v>0.7083333333333334</v>
       </c>
       <c r="G46">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I46">
-        <v>0.4000000000000001</v>
+        <v>0.7259259259259259</v>
       </c>
       <c r="J46">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -2274,10 +2274,10 @@
         <v>0</v>
       </c>
       <c r="I47">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J47">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="48" spans="1:10">
@@ -2306,10 +2306,10 @@
         <v>0</v>
       </c>
       <c r="I48">
-        <v>0.6083333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J48">
-        <v>0.7083333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="49" spans="1:10">
@@ -2338,10 +2338,10 @@
         <v>0</v>
       </c>
       <c r="I49">
-        <v>0.2</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J49">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="50" spans="1:10">
@@ -2370,7 +2370,7 @@
         <v>0</v>
       </c>
       <c r="I50">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J50">
         <v>0.75</v>
@@ -2402,7 +2402,7 @@
         <v>0</v>
       </c>
       <c r="I51">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J51">
         <v>0.75</v>
@@ -2434,7 +2434,7 @@
         <v>0</v>
       </c>
       <c r="I52">
-        <v>0.6</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J52">
         <v>0.75</v>
@@ -2460,16 +2460,16 @@
         <v>0.5833333333333334</v>
       </c>
       <c r="G53">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I53">
-        <v>0.6333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J53">
-        <v>0.7916666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -2492,16 +2492,16 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G54">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H54">
         <v>0.5</v>
       </c>
       <c r="I54">
-        <v>0.4000000000000001</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J54">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="55" spans="1:10">
@@ -2524,16 +2524,16 @@
         <v>0.625</v>
       </c>
       <c r="G55">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H55">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I55">
-        <v>0.4666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J55">
-        <v>0.5833333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="56" spans="1:10">
@@ -2562,10 +2562,10 @@
         <v>0.5</v>
       </c>
       <c r="I56">
-        <v>0.4000000000000001</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J56">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -2588,16 +2588,16 @@
         <v>0.75</v>
       </c>
       <c r="G57">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H57">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I57">
-        <v>0.4666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J57">
-        <v>0.5833333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2626,10 +2626,10 @@
         <v>0</v>
       </c>
       <c r="I58">
-        <v>0.7999999999999999</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J58">
-        <v>0.5833333333333334</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="59" spans="1:10">
@@ -2658,10 +2658,10 @@
         <v>0</v>
       </c>
       <c r="I59">
-        <v>0.4666666666666666</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J59">
-        <v>0.5833333333333334</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="60" spans="1:10">
@@ -2684,10 +2684,10 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="G60">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H60">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I60">
         <v>0.6</v>
@@ -2716,10 +2716,10 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="G61">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H61">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I61">
         <v>0.6</v>
@@ -2754,10 +2754,10 @@
         <v>0</v>
       </c>
       <c r="I62">
-        <v>0.5555555555555555</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="J62">
-        <v>0.5185185185185185</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
     <row r="63" spans="1:10">
@@ -2780,13 +2780,13 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H63">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I63">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="J63">
         <v>0.8571428571428571</v>
@@ -2812,10 +2812,10 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="G64">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H64">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="I64">
         <v>0.6</v>
@@ -2876,16 +2876,16 @@
         <v>0.7083333333333334</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H66">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I66">
-        <v>0.5</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J66">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="67" spans="1:10">
@@ -2914,10 +2914,10 @@
         <v>0.5</v>
       </c>
       <c r="I67">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J67">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -2940,16 +2940,16 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G68">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H68">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I68">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J68">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -3010,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="I70">
-        <v>0.625</v>
+        <v>0.5</v>
       </c>
       <c r="J70">
         <v>0.8333333333333334</v>
@@ -3068,10 +3068,10 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="G72">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="H72">
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="I72">
         <v>0.5</v>
@@ -3100,16 +3100,16 @@
         <v>0.625</v>
       </c>
       <c r="G73">
+        <v>1</v>
+      </c>
+      <c r="H73">
+        <v>1</v>
+      </c>
+      <c r="I73">
         <v>0.6666666666666666</v>
       </c>
-      <c r="H73">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="I73">
-        <v>0.4</v>
-      </c>
       <c r="J73">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="74" spans="1:10">
@@ -3138,10 +3138,10 @@
         <v>1</v>
       </c>
       <c r="I74">
-        <v>0.5333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J74">
-        <v>0.6666666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="75" spans="1:10">
@@ -3164,10 +3164,10 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G75">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H75">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I75">
         <v>0.6</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="I76">
-        <v>0.6</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J76">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="77" spans="1:10">
@@ -3234,10 +3234,10 @@
         <v>0</v>
       </c>
       <c r="I77">
-        <v>0.6</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J77">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="78" spans="1:10">
@@ -3266,10 +3266,10 @@
         <v>0</v>
       </c>
       <c r="I78">
-        <v>0.4000000000000001</v>
+        <v>0.7259259259259259</v>
       </c>
       <c r="J78">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="79" spans="1:10">
@@ -3298,10 +3298,10 @@
         <v>0</v>
       </c>
       <c r="I79">
-        <v>0.5666666666666667</v>
+        <v>0.7259259259259259</v>
       </c>
       <c r="J79">
-        <v>0.7083333333333334</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="80" spans="1:10">
@@ -3330,10 +3330,10 @@
         <v>0</v>
       </c>
       <c r="I80">
-        <v>0.8333333333333334</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J80">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="81" spans="1:10">
@@ -3362,10 +3362,10 @@
         <v>0</v>
       </c>
       <c r="I81">
-        <v>0.6</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J81">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="82" spans="1:10">
@@ -3388,16 +3388,16 @@
         <v>0.625</v>
       </c>
       <c r="G82">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I82">
-        <v>0.5</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J82">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="83" spans="1:10">
@@ -3426,10 +3426,10 @@
         <v>0</v>
       </c>
       <c r="I83">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J83">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="84" spans="1:10">
@@ -3458,10 +3458,10 @@
         <v>0</v>
       </c>
       <c r="I84">
-        <v>0.3333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="J84">
-        <v>0.4166666666666667</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="85" spans="1:10">
@@ -3490,10 +3490,10 @@
         <v>0</v>
       </c>
       <c r="I85">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J85">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -3516,16 +3516,16 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G86">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="H86">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I86">
-        <v>0.5</v>
+        <v>0.6999999999999998</v>
       </c>
       <c r="J86">
-        <v>0.625</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="87" spans="1:10">
@@ -3554,7 +3554,7 @@
         <v>0</v>
       </c>
       <c r="I87">
-        <v>0.8666666666666667</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J87">
         <v>0.75</v>
@@ -3586,10 +3586,10 @@
         <v>0</v>
       </c>
       <c r="I88">
-        <v>0.4000000000000001</v>
+        <v>0.5</v>
       </c>
       <c r="J88">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="89" spans="1:10">
@@ -3650,10 +3650,10 @@
         <v>0</v>
       </c>
       <c r="I90">
-        <v>0.7518518518518519</v>
+        <v>0.6</v>
       </c>
       <c r="J90">
-        <v>0.875</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="91" spans="1:10">
@@ -3682,10 +3682,10 @@
         <v>0</v>
       </c>
       <c r="I91">
-        <v>0.4666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J91">
-        <v>0.5833333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="92" spans="1:10">
@@ -3708,16 +3708,16 @@
         <v>0.6666666666666666</v>
       </c>
       <c r="G92">
-        <v>0.5</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="H92">
         <v>0.5</v>
       </c>
       <c r="I92">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J92">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="93" spans="1:10">
@@ -3746,10 +3746,10 @@
         <v>0</v>
       </c>
       <c r="I93">
-        <v>0.4666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J93">
-        <v>0.6666666666666666</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="94" spans="1:10">
@@ -3778,10 +3778,10 @@
         <v>0</v>
       </c>
       <c r="I94">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J94">
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="95" spans="1:10">
@@ -3804,10 +3804,10 @@
         <v>0.5</v>
       </c>
       <c r="G95">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H95">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I95">
         <v>0.6</v>
@@ -3836,16 +3836,16 @@
         <v>0.7083333333333334</v>
       </c>
       <c r="G96">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="H96">
-        <v>0.3333333333333333</v>
+        <v>0</v>
       </c>
       <c r="I96">
-        <v>0.6666666666666666</v>
+        <v>0.6</v>
       </c>
       <c r="J96">
-        <v>0.8333333333333334</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="97" spans="1:10">
@@ -3868,16 +3868,16 @@
         <v>0.5714285714285714</v>
       </c>
       <c r="G97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I97">
-        <v>0.4000000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="J97">
-        <v>0.5714285714285714</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="98" spans="1:10">
@@ -3900,16 +3900,16 @@
         <v>0.625</v>
       </c>
       <c r="G98">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H98">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="I98">
-        <v>0.6333333333333333</v>
+        <v>0.6</v>
       </c>
       <c r="J98">
-        <v>0.7916666666666666</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="99" spans="1:10">
@@ -3932,16 +3932,16 @@
         <v>0.75</v>
       </c>
       <c r="G99">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H99">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I99">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J99">
-        <v>0</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="100" spans="1:10">
@@ -3964,16 +3964,16 @@
         <v>0.7142857142857143</v>
       </c>
       <c r="G100">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H100">
         <v>1</v>
       </c>
       <c r="I100">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="J100">
-        <v>0.7142857142857143</v>
+        <v>0.8571428571428571</v>
       </c>
     </row>
     <row r="101" spans="1:10">
@@ -3996,16 +3996,16 @@
         <v>0.8333333333333334</v>
       </c>
       <c r="G101">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="H101">
-        <v>0.6666666666666666</v>
+        <v>0</v>
       </c>
       <c r="I101">
-        <v>0.4000000000000001</v>
+        <v>0.5185185185185185</v>
       </c>
       <c r="J101">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
   </sheetData>
@@ -4134,16 +4134,16 @@
         <v>0.7072222222222223</v>
       </c>
       <c r="C2">
-        <v>0.2913888888888889</v>
+        <v>0.1336666666666667</v>
       </c>
       <c r="D2">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F2">
-        <v>34</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4154,16 +4154,16 @@
         <v>0.715</v>
       </c>
       <c r="C3">
-        <v>0.2952777777777778</v>
+        <v>0.1475</v>
       </c>
       <c r="D3">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>38</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -4174,16 +4174,16 @@
         <v>0.5337777777777777</v>
       </c>
       <c r="C4">
-        <v>0.5265343915343915</v>
+        <v>0.6144074074074074</v>
       </c>
       <c r="D4">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E4">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -4194,16 +4194,16 @@
         <v>0.6837367724867724</v>
       </c>
       <c r="C5">
-        <v>0.6423809523809524</v>
+        <v>0.7806481481481481</v>
       </c>
       <c r="D5">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="F5">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -4244,22 +4244,22 @@
         <v>116</v>
       </c>
       <c r="B2">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="C2">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="D2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F2">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="G2">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -4267,22 +4267,22 @@
         <v>117</v>
       </c>
       <c r="B3">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C3">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="G3">
-        <v>59</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -4290,22 +4290,22 @@
         <v>118</v>
       </c>
       <c r="B4">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="C4">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="D4">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="E4">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="F4">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="G4">
-        <v>45</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -4313,22 +4313,22 @@
         <v>119</v>
       </c>
       <c r="B5">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D5">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="E5">
-        <v>37</v>
+        <v>63</v>
       </c>
       <c r="F5">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="G5">
-        <v>46</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>